<commit_message>
Split emergency contact into emergency_contact_name + emergency_contact_number
- Replace emergency_contact field with two separate fields:
  emergency_contact_name (Data) and emergency_contact_number (Data/Phone)
- Update Cohort 3 XLSX: rename column + add emergency_contact_name column
  (25/94 students have named emergency contacts from original form submissions)

https://claude.ai/code/session_01F4sDVWMLHGgtWJs3PzeGXU
</commit_message>
<xml_diff>
--- a/outputs/Cohort3_Student_Upload.xlsx
+++ b/outputs/Cohort3_Student_Upload.xlsx
@@ -547,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP95"/>
+  <dimension ref="A1:AQ95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -698,7 +698,7 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>emergency_contact</t>
+          <t>emergency_contact_number</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
@@ -799,6 +799,11 @@
       <c r="AP1" t="inlineStr">
         <is>
           <t>literacy_score</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>emergency_contact_name</t>
         </is>
       </c>
     </row>
@@ -960,6 +965,7 @@
       <c r="AO2" t="n">
         <v>40</v>
       </c>
+      <c r="AQ2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -1122,6 +1128,7 @@
       <c r="AP3" t="n">
         <v>75</v>
       </c>
+      <c r="AQ3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -1288,6 +1295,7 @@
       <c r="AP4" t="n">
         <v>80</v>
       </c>
+      <c r="AQ4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -1458,6 +1466,7 @@
       <c r="AP5" t="n">
         <v>70</v>
       </c>
+      <c r="AQ5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1628,6 +1637,11 @@
       <c r="AP6" t="n">
         <v>60</v>
       </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>Joseph Chileshe</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -1786,6 +1800,7 @@
       <c r="AP7" t="n">
         <v>90</v>
       </c>
+      <c r="AQ7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1951,6 +1966,11 @@
       </c>
       <c r="AP8" t="n">
         <v>60</v>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>Angel Phiri</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -2070,6 +2090,7 @@
       <c r="AP9" t="n">
         <v>80</v>
       </c>
+      <c r="AQ9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -2236,6 +2257,7 @@
       <c r="AP10" t="n">
         <v>70</v>
       </c>
+      <c r="AQ10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -2402,6 +2424,7 @@
       <c r="AP11" t="n">
         <v>60</v>
       </c>
+      <c r="AQ11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -2568,6 +2591,7 @@
       <c r="AP12" t="n">
         <v>95</v>
       </c>
+      <c r="AQ12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -2730,6 +2754,7 @@
       <c r="AP13" t="n">
         <v>85</v>
       </c>
+      <c r="AQ13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -2896,6 +2921,11 @@
       <c r="AP14" t="n">
         <v>60</v>
       </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>Killian Bbindu</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -3049,6 +3079,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -3211,6 +3242,11 @@
       <c r="AP16" t="n">
         <v>85</v>
       </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>Dickson Banda</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -3373,6 +3409,7 @@
       <c r="AP17" t="n">
         <v>40</v>
       </c>
+      <c r="AQ17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -3535,6 +3572,7 @@
       <c r="AP18" t="n">
         <v>95</v>
       </c>
+      <c r="AQ18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -3695,6 +3733,7 @@
       <c r="AN19" t="n">
         <v>93</v>
       </c>
+      <c r="AQ19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -3865,6 +3904,7 @@
       <c r="AP20" t="n">
         <v>65</v>
       </c>
+      <c r="AQ20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -4018,6 +4058,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -4175,6 +4216,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -4349,6 +4391,11 @@
       <c r="AP23" t="n">
         <v>50</v>
       </c>
+      <c r="AQ23" t="inlineStr">
+        <is>
+          <t>Constance Mulowa</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -4511,6 +4558,7 @@
       <c r="AP24" t="n">
         <v>80</v>
       </c>
+      <c r="AQ24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -4673,6 +4721,11 @@
       <c r="AP25" t="n">
         <v>85</v>
       </c>
+      <c r="AQ25" t="inlineStr">
+        <is>
+          <t>Angela</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -4838,6 +4891,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -5004,6 +5058,7 @@
       <c r="AP27" t="n">
         <v>90</v>
       </c>
+      <c r="AQ27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -5166,6 +5221,11 @@
       <c r="AP28" t="n">
         <v>60</v>
       </c>
+      <c r="AQ28" t="inlineStr">
+        <is>
+          <t>Melon Mwansa</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -5336,6 +5396,7 @@
       <c r="AP29" t="n">
         <v>60</v>
       </c>
+      <c r="AQ29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -5496,6 +5557,7 @@
       <c r="AN30" t="n">
         <v>55</v>
       </c>
+      <c r="AQ30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -5654,6 +5716,7 @@
       <c r="AP31" t="n">
         <v>60</v>
       </c>
+      <c r="AQ31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -5812,6 +5875,7 @@
       <c r="AP32" t="n">
         <v>85</v>
       </c>
+      <c r="AQ32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -5978,6 +6042,7 @@
       <c r="AP33" t="n">
         <v>60</v>
       </c>
+      <c r="AQ33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -6139,6 +6204,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -6301,6 +6367,7 @@
       <c r="AP35" t="n">
         <v>40</v>
       </c>
+      <c r="AQ35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -6394,6 +6461,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -6555,6 +6623,11 @@
       </c>
       <c r="AP37" t="n">
         <v>90</v>
+      </c>
+      <c r="AQ37" t="inlineStr">
+        <is>
+          <t>Faith</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -6674,6 +6747,7 @@
       <c r="AP38" t="n">
         <v>50</v>
       </c>
+      <c r="AQ38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -6827,6 +6901,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -6997,6 +7072,7 @@
       <c r="AP40" t="n">
         <v>70</v>
       </c>
+      <c r="AQ40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -7159,6 +7235,7 @@
       <c r="AP41" t="n">
         <v>60</v>
       </c>
+      <c r="AQ41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -7318,6 +7395,7 @@
       <c r="AP42" t="n">
         <v>85</v>
       </c>
+      <c r="AQ42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -7488,6 +7566,11 @@
       <c r="AP43" t="n">
         <v>85</v>
       </c>
+      <c r="AQ43" t="inlineStr">
+        <is>
+          <t>Mercy Mpundu</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -7658,6 +7741,7 @@
       <c r="AP44" t="n">
         <v>85</v>
       </c>
+      <c r="AQ44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -7811,6 +7895,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -7977,6 +8062,11 @@
       <c r="AP46" t="n">
         <v>85</v>
       </c>
+      <c r="AQ46" t="inlineStr">
+        <is>
+          <t>Kondwani Gondwe</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -8139,6 +8229,7 @@
       <c r="AP47" t="n">
         <v>75</v>
       </c>
+      <c r="AQ47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -8232,6 +8323,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -8402,6 +8494,7 @@
       <c r="AP49" t="n">
         <v>75</v>
       </c>
+      <c r="AQ49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -8559,6 +8652,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -8729,6 +8823,7 @@
       <c r="AP51" t="n">
         <v>70</v>
       </c>
+      <c r="AQ51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -8891,6 +8986,7 @@
       <c r="AP52" t="n">
         <v>35</v>
       </c>
+      <c r="AQ52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -9043,6 +9139,7 @@
       <c r="AN53" t="n">
         <v>147</v>
       </c>
+      <c r="AQ53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
@@ -9213,6 +9310,7 @@
       <c r="AP54" t="n">
         <v>35</v>
       </c>
+      <c r="AQ54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -9375,6 +9473,11 @@
       <c r="AP55" t="n">
         <v>80</v>
       </c>
+      <c r="AQ55" t="inlineStr">
+        <is>
+          <t>Josiah</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
@@ -9531,6 +9634,7 @@
       <c r="AN56" t="n">
         <v>48</v>
       </c>
+      <c r="AQ56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -9684,6 +9788,11 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ57" t="inlineStr">
+        <is>
+          <t>Josiah</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
@@ -9836,6 +9945,7 @@
       <c r="AN58" t="n">
         <v>5</v>
       </c>
+      <c r="AQ58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -10007,6 +10117,11 @@
       <c r="AP59" t="n">
         <v>60</v>
       </c>
+      <c r="AQ59" t="inlineStr">
+        <is>
+          <t>Alice Nakamba</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
@@ -10169,6 +10284,7 @@
       <c r="AP60" t="n">
         <v>15</v>
       </c>
+      <c r="AQ60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -10327,6 +10443,7 @@
       <c r="AP61" t="n">
         <v>65</v>
       </c>
+      <c r="AQ61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
@@ -10491,6 +10608,7 @@
       <c r="AN62" t="n">
         <v>23</v>
       </c>
+      <c r="AQ62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -10657,6 +10775,11 @@
       <c r="AP63" t="n">
         <v>85</v>
       </c>
+      <c r="AQ63" t="inlineStr">
+        <is>
+          <t>Elizabeth Phiri</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -10823,6 +10946,7 @@
       <c r="AP64" t="n">
         <v>85</v>
       </c>
+      <c r="AQ64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -10985,6 +11109,7 @@
       <c r="AP65" t="n">
         <v>55</v>
       </c>
+      <c r="AQ65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
@@ -11141,6 +11266,7 @@
       <c r="AN66" t="n">
         <v>2</v>
       </c>
+      <c r="AQ66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -11303,6 +11429,11 @@
       <c r="AP67" t="n">
         <v>40</v>
       </c>
+      <c r="AQ67" t="inlineStr">
+        <is>
+          <t>Chola Nkhoma</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
@@ -11468,6 +11599,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -11626,6 +11758,11 @@
       <c r="AP69" t="n">
         <v>70</v>
       </c>
+      <c r="AQ69" t="inlineStr">
+        <is>
+          <t>Rabcca Mulenga</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -11792,6 +11929,7 @@
       <c r="AP70" t="n">
         <v>60</v>
       </c>
+      <c r="AQ70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -11962,6 +12100,7 @@
       <c r="AP71" t="n">
         <v>85</v>
       </c>
+      <c r="AQ71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -12132,6 +12271,11 @@
       <c r="AP72" t="n">
         <v>65</v>
       </c>
+      <c r="AQ72" t="inlineStr">
+        <is>
+          <t>Moses Mubita</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -12295,6 +12439,11 @@
       </c>
       <c r="AN73" t="n">
         <v>91</v>
+      </c>
+      <c r="AQ73" t="inlineStr">
+        <is>
+          <t>Mercy Mpundu</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -12414,6 +12563,7 @@
       <c r="AP74" t="n">
         <v>50</v>
       </c>
+      <c r="AQ74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -12579,6 +12729,11 @@
       </c>
       <c r="AP75" t="n">
         <v>90</v>
+      </c>
+      <c r="AQ75" t="inlineStr">
+        <is>
+          <t>Ireen Munzele Siwela</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -12673,6 +12828,11 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ76" t="inlineStr">
+        <is>
+          <t>Mercy Mpundu</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -12838,6 +12998,11 @@
       <c r="AN77" t="n">
         <v>94</v>
       </c>
+      <c r="AQ77" t="inlineStr">
+        <is>
+          <t>Isabel Nyundu</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
@@ -13005,6 +13170,7 @@
       <c r="AP78" t="n">
         <v>90</v>
       </c>
+      <c r="AQ78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -13171,6 +13337,7 @@
       <c r="AP79" t="n">
         <v>65</v>
       </c>
+      <c r="AQ79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
@@ -13335,6 +13502,7 @@
       <c r="AN80" t="n">
         <v>102</v>
       </c>
+      <c r="AQ80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -13501,6 +13669,7 @@
       <c r="AP81" t="n">
         <v>75</v>
       </c>
+      <c r="AQ81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
@@ -13671,6 +13840,11 @@
       <c r="AP82" t="n">
         <v>100</v>
       </c>
+      <c r="AQ82" t="inlineStr">
+        <is>
+          <t>Oswell Kangwa</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -13829,6 +14003,7 @@
       <c r="AP83" t="n">
         <v>70</v>
       </c>
+      <c r="AQ83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
@@ -14003,6 +14178,7 @@
       <c r="AP84" t="n">
         <v>80</v>
       </c>
+      <c r="AQ84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -14160,6 +14336,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
@@ -14329,6 +14506,11 @@
       </c>
       <c r="AP86" t="n">
         <v>85</v>
+      </c>
+      <c r="AQ86" t="inlineStr">
+        <is>
+          <t>Mable Bweupe</t>
+        </is>
       </c>
     </row>
     <row r="87">
@@ -14423,6 +14605,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
@@ -14580,6 +14763,7 @@
           <t>Path A</t>
         </is>
       </c>
+      <c r="AQ88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -14743,6 +14927,7 @@
       <c r="AO89" t="n">
         <v>55</v>
       </c>
+      <c r="AQ89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
@@ -14905,6 +15090,11 @@
       <c r="AP90" t="n">
         <v>60</v>
       </c>
+      <c r="AQ90" t="inlineStr">
+        <is>
+          <t>Tassy Mulenga</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -15067,6 +15257,7 @@
       <c r="AP91" t="n">
         <v>85</v>
       </c>
+      <c r="AQ91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
@@ -15237,6 +15428,7 @@
       <c r="AP92" t="n">
         <v>70</v>
       </c>
+      <c r="AQ92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -15400,6 +15592,11 @@
       <c r="AO93" t="n">
         <v>80</v>
       </c>
+      <c r="AQ93" t="inlineStr">
+        <is>
+          <t>Justina Weza</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
@@ -15570,6 +15767,7 @@
       <c r="AP94" t="n">
         <v>70</v>
       </c>
+      <c r="AQ94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -15736,6 +15934,7 @@
       <c r="AP95" t="n">
         <v>45</v>
       </c>
+      <c r="AQ95" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>